<commit_message>
Update Task Tracker + Hard Milestones from full mailbox review (7 Aug): close 3 tasks, add 9 new, flag contractual-date gap
</commit_message>
<xml_diff>
--- a/260807_K5M_Project Management_Tasks and Calendar.xlsx
+++ b/260807_K5M_Project Management_Tasks and Calendar.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$5:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Task Tracker'!$A$10:$L$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Task Tracker'!$A$10:$K$67</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -732,6 +732,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2974,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="47" min="1" max="1"/>
@@ -4789,13 +4795,13 @@
       <c r="H45" s="78" t="n"/>
       <c r="I45" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J45" s="75" t="n"/>
       <c r="K45" s="78" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire — decided today to extend this to a 2-day effort (was previously a single 31 Aug entry). Calendar Hard Milestone updated accordingly. Site visit timing under ambiguity as of the 3 Aug BOQ gap meeting — regardless, need white-box photos ready and a post-site-survey deliverable prepared.</t>
+          <t>Per 4 Aug meeting with Claire — decided today to extend this to a 2-day effort (was previously a single 31 Aug entry). Calendar Hard Milestone updated accordingly. Site visit timing under ambiguity as of the 3 Aug BOQ gap meeting — regardless, need white-box photos ready and a post-site-survey deliverable prepared. Update 7 Aug: this is now a settled decision, not just under review — re-scoped from a technical review to a client-facing "show face" meeting, relying on the site team (not a technical review team) for measurements.</t>
         </is>
       </c>
       <c r="L45" s="93">
@@ -4985,13 +4991,13 @@
       <c r="H49" s="78" t="n"/>
       <c r="I49" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J49" s="75" t="n"/>
       <c r="K49" s="78" t="inlineStr">
         <is>
-          <t>Per 3 Aug BOQ gap meeting decision (b). Filippo Sona is WDCO's co-founder and main partner — internal, not client-facing.</t>
+          <t>Per 3 Aug BOQ gap meeting decision (b). Filippo Sona is WDCO's co-founder and main partner — internal, not client-facing. Done — sent 6 Aug ("K5M | BOQ Gap / Variables since Kick Off"), confirmed via mailbox review 7 Aug.</t>
         </is>
       </c>
       <c r="L49" s="93">
@@ -5034,13 +5040,13 @@
       <c r="H50" s="78" t="n"/>
       <c r="I50" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J50" s="75" t="n"/>
       <c r="K50" s="78" t="inlineStr">
         <is>
-          <t>Per 3 Aug BOQ gap meeting decision (c). Maria is WDCO's logistics personnel, handling container booking etc.</t>
+          <t>Per 3 Aug BOQ gap meeting decision (c). Maria is WDCO's logistics personnel, handling container booking etc. Done — sent 7 Aug to Maria Al Balushi with real numbers: ~30 pieces for one room, target departure window 5-10 Oct, 10 Oct hard deadline. Full weight/size estimate still promised for end of August.</t>
         </is>
       </c>
       <c r="L50" s="93">
@@ -5177,7 +5183,7 @@
       <c r="H53" s="78" t="n"/>
       <c r="I53" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J53" s="87" t="n">
@@ -5185,7 +5191,7 @@
       </c>
       <c r="K53" s="78" t="inlineStr">
         <is>
-          <t>Per 3 Aug BOQ gap meeting decision (f). Deadline of 7 Aug confirmed by Ariel.</t>
+          <t>Per 3 Aug BOQ gap meeting decision (f). Deadline of 7 Aug confirmed by Ariel. Done — Ariel delivered A4 layout drawings via WeTransfer, 7 Aug.</t>
         </is>
       </c>
       <c r="L53" s="93">
@@ -5430,9 +5436,421 @@
         <v/>
       </c>
     </row>
-    <row r="59"/>
+    <row r="59">
+      <c r="A59" s="94" t="n">
+        <v>49</v>
+      </c>
+      <c r="B59" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C59" s="95" t="inlineStr">
+        <is>
+          <t>Reconcile the internal working schedule against the actual contractual mock-up deadline (30 Nov 2026, per the original award letter) with Filippo/Claire — the internal schedule appears to have drifted past it</t>
+        </is>
+      </c>
+      <c r="D59" s="95" t="inlineStr">
+        <is>
+          <t>Contractual - Client Facing</t>
+        </is>
+      </c>
+      <c r="E59" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="95" t="inlineStr">
+        <is>
+          <t>Meeting online</t>
+        </is>
+      </c>
+      <c r="G59" s="95" t="inlineStr">
+        <is>
+          <t>Filippo Sona</t>
+        </is>
+      </c>
+      <c r="H59" s="95" t="inlineStr">
+        <is>
+          <t>Claire</t>
+        </is>
+      </c>
+      <c r="I59" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J59" s="94" t="n"/>
+      <c r="K59" s="95" t="inlineStr">
+        <is>
+          <t>Surfaced via full mailbox review, 7 Aug. Filippo cited 30 Nov as the hard contractual milestone in a live liability-negotiation email with the client; internal planning has since referenced 20 Dec. Needs reconciling, not just tracking forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="94" t="n">
+        <v>50</v>
+      </c>
+      <c r="B60" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C60" s="95" t="inlineStr">
+        <is>
+          <t>Chase H&amp;T on the sample box (due 8 Aug) — escalate per the Plan-B threat already given if it slips</t>
+        </is>
+      </c>
+      <c r="D60" s="95" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="E60" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G60" s="95" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H60" s="95" t="n"/>
+      <c r="I60" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J60" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K60" s="95" t="inlineStr">
+        <is>
+          <t>Shagun already put H&amp;T on notice 6 Aug: if the 8 Aug date can't be held, escalate to management and source samples elsewhere, with H&amp;T then required to match approved samples exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="94" t="n">
+        <v>51</v>
+      </c>
+      <c r="B61" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C61" s="95" t="inlineStr">
+        <is>
+          <t>Confirm H&amp;T has remade the metal samples produced in the wrong size</t>
+        </is>
+      </c>
+      <c r="D61" s="95" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="E61" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G61" s="95" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H61" s="95" t="n"/>
+      <c r="I61" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J61" s="94" t="n"/>
+      <c r="K61" s="95" t="inlineStr">
+        <is>
+          <t>Flagged 6 Aug — metal samples came back in the wrong dimensions against the confirmed sizes (Fabric/Wood/Glass 14x10cm, Metal 10x7cm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="94" t="n">
+        <v>52</v>
+      </c>
+      <c r="B62" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C62" s="95" t="inlineStr">
+        <is>
+          <t>Follow up with Adil Mokaddem on the corrupted/incomplete DWG file (plan numbers ET01-T1B1-SDB-100 through 150)</t>
+        </is>
+      </c>
+      <c r="D62" s="95" t="inlineStr">
+        <is>
+          <t>RFI - Client</t>
+        </is>
+      </c>
+      <c r="E62" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G62" s="95" t="inlineStr">
+        <is>
+          <t>Adil</t>
+        </is>
+      </c>
+      <c r="H62" s="95" t="n"/>
+      <c r="I62" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J62" s="94" t="n"/>
+      <c r="K62" s="95" t="inlineStr">
+        <is>
+          <t>RFI sent 7 Aug ("WDCO K5M | PH T1B1 | RFI | Problem with DWG File"); architect's fix still pending as of the mailbox review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="94" t="n">
+        <v>53</v>
+      </c>
+      <c r="B63" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C63" s="95" t="inlineStr">
+        <is>
+          <t>Follow up with Adil Mokaddem on structural reinforcement provisions for the fit-out (ceiling supports/backing around wardrobe and fitted-sofa areas), incl. recent site photos</t>
+        </is>
+      </c>
+      <c r="D63" s="95" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="E63" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G63" s="95" t="inlineStr">
+        <is>
+          <t>Adil</t>
+        </is>
+      </c>
+      <c r="H63" s="95" t="n"/>
+      <c r="I63" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J63" s="94" t="n"/>
+      <c r="K63" s="95" t="inlineStr">
+        <is>
+          <t>Requested 4 Aug, no reply captured as of 7 Aug mailbox review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="94" t="n">
+        <v>54</v>
+      </c>
+      <c r="B64" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C64" s="95" t="inlineStr">
+        <is>
+          <t>Confirm wall art specification and art-consultant point of contact with the client</t>
+        </is>
+      </c>
+      <c r="D64" s="95" t="inlineStr">
+        <is>
+          <t>RFI - Client</t>
+        </is>
+      </c>
+      <c r="E64" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G64" s="95" t="inlineStr">
+        <is>
+          <t>Abdellatif Menbar</t>
+        </is>
+      </c>
+      <c r="H64" s="95" t="n"/>
+      <c r="I64" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J64" s="94" t="n"/>
+      <c r="K64" s="95" t="inlineStr">
+        <is>
+          <t>Requested 6 Aug, referencing G&amp;B's earlier advice to coordinate with the project's art consultant — contact still unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="94" t="n">
+        <v>55</v>
+      </c>
+      <c r="B65" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C65" s="95" t="inlineStr">
+        <is>
+          <t>Raise the PO for Ariel's drafting invoice (USD 720, 72 pages reformatted to A4)</t>
+        </is>
+      </c>
+      <c r="D65" s="95" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E65" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" s="95" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G65" s="95" t="inlineStr">
+        <is>
+          <t>Ariel</t>
+        </is>
+      </c>
+      <c r="H65" s="95" t="n"/>
+      <c r="I65" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J65" s="94" t="n"/>
+      <c r="K65" s="95" t="inlineStr">
+        <is>
+          <t>Quote accepted in principle 4 Aug; PO not yet raised as of 7 Aug mailbox review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="94" t="n">
+        <v>56</v>
+      </c>
+      <c r="B66" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C66" s="95" t="inlineStr">
+        <is>
+          <t>Track H&amp;T capacity/responsiveness risk — factory completion now flagged for 16 Aug (was believed already in preparation), competing for capacity against another WDCO project (2576-F)</t>
+        </is>
+      </c>
+      <c r="D66" s="95" t="inlineStr">
+        <is>
+          <t>Communication Management - Production Partner</t>
+        </is>
+      </c>
+      <c r="E66" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="95" t="inlineStr">
+        <is>
+          <t>Meeting online</t>
+        </is>
+      </c>
+      <c r="G66" s="95" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H66" s="95" t="n"/>
+      <c r="I66" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J66" s="94" t="n"/>
+      <c r="K66" s="95" t="inlineStr">
+        <is>
+          <t>Khamille's high-importance flag, 7 Aug: "the dates and info we're getting keep shifting, and it's getting hard to plan around." Same underlying H&amp;T issue as the sample-box escalation above — treat together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="94" t="n">
+        <v>57</v>
+      </c>
+      <c r="B67" s="94" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C67" s="95" t="inlineStr">
+        <is>
+          <t>Check resolution status of the table stability defect on T1B1-BR-CG-03 (base too narrow, CTO recommended ≥36cm base)</t>
+        </is>
+      </c>
+      <c r="D67" s="95" t="inlineStr">
+        <is>
+          <t>FFE SHD</t>
+        </is>
+      </c>
+      <c r="E67" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" s="95" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G67" s="95" t="inlineStr">
+        <is>
+          <t>Fabrizio</t>
+        </is>
+      </c>
+      <c r="H67" s="95" t="n"/>
+      <c r="I67" s="94" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J67" s="94" t="n"/>
+      <c r="K67" s="95" t="inlineStr">
+        <is>
+          <t>Flagged by Fabrizio Pensalfini in mid-July; resolution status not visible in the mailbox review — worth a direct check.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:L58"/>
+  <autoFilter ref="A10:K67"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>
@@ -9964,7 +10382,7 @@
       </c>
       <c r="U10" s="17" t="inlineStr">
         <is>
-          <t>Must reach WDCO Dubai by 10 Aug.</t>
+          <t>Must reach WDCO Dubai by 10 Aug. (#50) Shagun has put H&amp;T on notice: management escalation + Plan-B sourcing if this slips.</t>
         </is>
       </c>
     </row>
@@ -10429,7 +10847,7 @@
       </c>
       <c r="U20" s="17" t="inlineStr">
         <is>
-          <t>Indicative revised readiness date.</t>
+          <t>Indicative revised readiness date — later than the actual contractual milestone (30 Nov, see row above). (#49) Needs reconciling with Filippo/Claire.</t>
         </is>
       </c>
     </row>
@@ -10552,6 +10970,72 @@
       <c r="U22" s="17" t="inlineStr">
         <is>
           <t>Agenda: see meetings/260803_K5M_Meeting_BOQ_Scope_Gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" s="28">
+      <c r="R23" s="17" t="inlineStr">
+        <is>
+          <t>30 Nov 2026</t>
+        </is>
+      </c>
+      <c r="S23" s="17" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="T23" s="17" t="inlineStr">
+        <is>
+          <t>T1B1 mock-up contractual deadline</t>
+        </is>
+      </c>
+      <c r="U23" s="17" t="inlineStr">
+        <is>
+          <t>(#49) Hard contractual milestone per the original award letter, cited by Filippo Sona 6 Aug — fully completed, installed, ready for review/approval. Predates and is earlier than the 20 Dec indicative date below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1" s="28">
+      <c r="R24" s="17" t="inlineStr">
+        <is>
+          <t>10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="S24" s="17" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="T24" s="17" t="inlineStr">
+        <is>
+          <t>Container shipment hard deadline</t>
+        </is>
+      </c>
+      <c r="U24" s="17" t="inlineStr">
+        <is>
+          <t>(#40) Confirmed 7 Aug with Maria Al Balushi — target departure window 5-10 Oct, ~30 pieces for one room. Full weight/size estimate still due end of August.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" s="28">
+      <c r="R25" s="17" t="inlineStr">
+        <is>
+          <t>16 Aug 2026</t>
+        </is>
+      </c>
+      <c r="S25" s="17" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="T25" s="17" t="inlineStr">
+        <is>
+          <t>K5M factory materials completion (flagged risk)</t>
+        </is>
+      </c>
+      <c r="U25" s="17" t="inlineStr">
+        <is>
+          <t>(#56) Khamille's high-importance flag, 7 Aug — previously understood to be already in preparation. Coincides with Material Package Fitout's own 10-day sample turnaround target.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
#totalcheck: Woody upkeep on Tasks 30, 31, 44 from email cross-check
</commit_message>
<xml_diff>
--- a/260807_K5M_Project Management_Tasks and Calendar.xlsx
+++ b/260807_K5M_Project Management_Tasks and Calendar.xlsx
@@ -4544,13 +4544,13 @@
       <c r="H40" s="78" t="n"/>
       <c r="I40" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J40" s="75" t="n"/>
       <c r="K40" s="78" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire: Paris design team clarified 3 coating finishes look similar but are different codes based on metal nature — doesn't align with VE. Agreed to proceed via H&amp;T China team using client visual references rather than resolving the code discrepancy first.</t>
+          <t>Per 4 Aug meeting with Claire: Paris design team clarified 3 coating finishes look similar but are different codes based on metal nature — doesn't align with VE. Agreed to proceed via H&amp;T China team using client visual references rather than resolving the code discrepancy first. Update 7 Aug: H&amp;T did start — metal samples came back in the wrong size, need remaking (see Task 51).</t>
         </is>
       </c>
       <c r="L40" s="93">
@@ -4597,13 +4597,13 @@
       </c>
       <c r="I41" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J41" s="75" t="n"/>
       <c r="K41" s="78" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire — fit-out drawings must be updated before scope can float further. Resti (Head of Engineering, joined this week) copied to stay informed.</t>
+          <t>Per 4 Aug meeting with Claire — fit-out drawings must be updated before scope can float further. Resti (Head of Engineering, joined this week) copied to stay informed. Update 7 Aug: Ariel confirmed receipt of 72 A1 pages, quoted USD 720 to reformat to A4, delivered 7 Aug (see Task 43, Done).</t>
         </is>
       </c>
       <c r="L41" s="93">
@@ -5230,7 +5230,7 @@
       <c r="H54" s="78" t="n"/>
       <c r="I54" s="75" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J54" s="87" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="K54" s="78" t="inlineStr">
         <is>
-          <t>Per 3 Aug BOQ gap meeting decision (j). Going forward, SHD review meeting minutes will be traced via the Shop Drawing Tracker itself rather than a separate MOM doc — content for this specific MOM still pending from Shagun as of 6 Aug.</t>
+          <t>Per 3 Aug BOQ gap meeting decision (j). Going forward, SHD review meeting minutes will be traced via the Shop Drawing Tracker itself rather than a separate MOM doc — content for this specific MOM still pending from Shagun as of 6 Aug. Done — sent 7 Aug (one day late) via the recurring "ProjectK5M: Internal Meeting Minutes" email, which also carried the site-visit re-scoping decision.</t>
         </is>
       </c>
       <c r="L54" s="93">

</xml_diff>